<commit_message>
feat: add front-end dashboard with stock portfolio visualization, sorting, and data import support
</commit_message>
<xml_diff>
--- a/assets/stocks.xlsx
+++ b/assets/stocks.xlsx
@@ -761,7 +761,7 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IBULPP-E1.NS</t>
+          <t>SAMMAANCAP.NS</t>
         </is>
       </c>
       <c r="B27" t="n">
@@ -839,7 +839,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>SHREEREF-M.NS</t>
+          <t>SHREEREF.BO</t>
         </is>
       </c>
       <c r="B33" t="n">
@@ -852,7 +852,7 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>SUPREMEPWR-ST.NS</t>
+          <t>SUPREMEPWR.NS</t>
         </is>
       </c>
       <c r="B34" t="n">

</xml_diff>